<commit_message>
Add new feature definitions for various sights and silencers in the mercenary compendium
</commit_message>
<xml_diff>
--- a/sources/compendium/merc-compendium.xlsx
+++ b/sources/compendium/merc-compendium.xlsx
@@ -1,24 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerom\Downloads\FoundryVTT-WindowsPortable-13.351\Data\systems\merc\sources\compendium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0737263E-F788-41AB-A910-41CCF7525933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0E6C67-2FDA-42BB-9D4A-3785E3A53F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Munition" sheetId="1" r:id="rId1"/>
     <sheet name="Weapon" sheetId="3" r:id="rId2"/>
-    <sheet name="Data Balistique" sheetId="5" state="hidden" r:id="rId3"/>
+    <sheet name="Feature" sheetId="6" r:id="rId3"/>
+    <sheet name="Armor" sheetId="7" r:id="rId4"/>
+    <sheet name="Equipement" sheetId="8" r:id="rId5"/>
+    <sheet name="Data Balistique" sheetId="5" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data Balistique'!$A$1:$AU$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Data Balistique'!$A$1:$AU$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Munition!$A$1:$M$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Weapon!$A$1:$AJ$383</definedName>
   </definedNames>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3445" uniqueCount="868">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3784" uniqueCount="1069">
   <si>
     <t>Munition</t>
   </si>
@@ -2645,6 +2648,609 @@
   </si>
   <si>
     <t>Indice de freinage Munition (1/m)</t>
+  </si>
+  <si>
+    <t>type feature</t>
+  </si>
+  <si>
+    <t>Bonus tir porté courte</t>
+  </si>
+  <si>
+    <t>Reduction de bruit</t>
+  </si>
+  <si>
+    <t>Reduction de bruit Latérale</t>
+  </si>
+  <si>
+    <t>Augmentation de longueur</t>
+  </si>
+  <si>
+    <t>Rarete</t>
+  </si>
+  <si>
+    <t>Prix</t>
+  </si>
+  <si>
+    <t>Poids (kg)</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Visée rudimentaire</t>
+  </si>
+  <si>
+    <t>pointeur Laser jour</t>
+  </si>
+  <si>
+    <t>Pointeur laser Nuit</t>
+  </si>
+  <si>
+    <t>Pointeur mixte</t>
+  </si>
+  <si>
+    <t>Viseur Holographique</t>
+  </si>
+  <si>
+    <t>Visée lunette</t>
+  </si>
+  <si>
+    <t>Aimpoint x2</t>
+  </si>
+  <si>
+    <t>Lunette IL x10</t>
+  </si>
+  <si>
+    <t>Lunette IL x16</t>
+  </si>
+  <si>
+    <t>Lunette IL x3</t>
+  </si>
+  <si>
+    <t>Lunette IL x4</t>
+  </si>
+  <si>
+    <t>Lunette IL x6</t>
+  </si>
+  <si>
+    <t>Lunette Jour x16</t>
+  </si>
+  <si>
+    <t>Lunette Jour x2,5-6</t>
+  </si>
+  <si>
+    <t>Lunette jour x4</t>
+  </si>
+  <si>
+    <t>Lunette Jour x4-16</t>
+  </si>
+  <si>
+    <t>Lunette Jour x6-24</t>
+  </si>
+  <si>
+    <t>Lunette Jour x7-35</t>
+  </si>
+  <si>
+    <t>Lunette Jour x5-30</t>
+  </si>
+  <si>
+    <t>Lunette mixte x3-15</t>
+  </si>
+  <si>
+    <t>Lunette Thermique x3</t>
+  </si>
+  <si>
+    <t>Lunette Thermique x10</t>
+  </si>
+  <si>
+    <t>Addons</t>
+  </si>
+  <si>
+    <t>Adaptateur Thermique</t>
+  </si>
+  <si>
+    <t>à mettre devant un Viseur Holo, permet le tir lunette</t>
+  </si>
+  <si>
+    <t>Loupe Jour Basculante x3</t>
+  </si>
+  <si>
+    <t>Silencieux</t>
+  </si>
+  <si>
+    <t>Csilint</t>
+  </si>
+  <si>
+    <t>Silencieux civil Léger</t>
+  </si>
+  <si>
+    <t>pour armes de poings</t>
+  </si>
+  <si>
+    <t>Silencieux civil Lourd</t>
+  </si>
+  <si>
+    <t>Calibres de .22 à 9x19</t>
+  </si>
+  <si>
+    <t>Silencieux civil Auto</t>
+  </si>
+  <si>
+    <t>calibres de .222 à .308</t>
+  </si>
+  <si>
+    <t>Silencieux militaire Léger</t>
+  </si>
+  <si>
+    <t>Silencieux militaire Lourd</t>
+  </si>
+  <si>
+    <t>calibres de .223 à .338</t>
+  </si>
+  <si>
+    <t>Silencieux militaire Auto</t>
+  </si>
+  <si>
+    <t>Calibres de 5,56 à 9mm pour armes automatiques</t>
+  </si>
+  <si>
+    <t>nom</t>
+  </si>
+  <si>
+    <t>Bonus tir porté moyenne</t>
+  </si>
+  <si>
+    <t>Bonus tir porté longue</t>
+  </si>
+  <si>
+    <t>Bonus tir porté extreme</t>
+  </si>
+  <si>
+    <t>crane</t>
+  </si>
+  <si>
+    <t>visage</t>
+  </si>
+  <si>
+    <t>cou</t>
+  </si>
+  <si>
+    <t>poitrine_gch</t>
+  </si>
+  <si>
+    <t>poitrine_dr</t>
+  </si>
+  <si>
+    <t>abdomen_gch</t>
+  </si>
+  <si>
+    <t>abdomen_dr</t>
+  </si>
+  <si>
+    <t>bas_ventre</t>
+  </si>
+  <si>
+    <t>bras_gch</t>
+  </si>
+  <si>
+    <t>bras_dr</t>
+  </si>
+  <si>
+    <t>av_bras_gch</t>
+  </si>
+  <si>
+    <t>av_bras_dr</t>
+  </si>
+  <si>
+    <t>main_gch</t>
+  </si>
+  <si>
+    <t>main_dr</t>
+  </si>
+  <si>
+    <t>cuisse_gch</t>
+  </si>
+  <si>
+    <t>cuisse_dr</t>
+  </si>
+  <si>
+    <t>jambe_gch</t>
+  </si>
+  <si>
+    <t>jambe_dr</t>
+  </si>
+  <si>
+    <t>pied_gch</t>
+  </si>
+  <si>
+    <t>pied_dr</t>
+  </si>
+  <si>
+    <t>Armures\Gilets</t>
+  </si>
+  <si>
+    <t>Gilet souple NIJ I</t>
+  </si>
+  <si>
+    <t>common</t>
+  </si>
+  <si>
+    <t>Gilet souple NIJ IIA</t>
+  </si>
+  <si>
+    <t>Gilet souple NIJ II</t>
+  </si>
+  <si>
+    <t>Gilet souple NIJ IIIA</t>
+  </si>
+  <si>
+    <t>uncommon</t>
+  </si>
+  <si>
+    <t>Gilet tactique NIJ IIIA + cervical</t>
+  </si>
+  <si>
+    <t>IOTV Gen III (soft + plaques ESAPI)</t>
+  </si>
+  <si>
+    <t>Dragon Skin SOV-3000</t>
+  </si>
+  <si>
+    <t>rare</t>
+  </si>
+  <si>
+    <t>Combinaison de protection CBRN</t>
+  </si>
+  <si>
+    <t>Armures\Casques</t>
+  </si>
+  <si>
+    <t>Casque lourd PASGT</t>
+  </si>
+  <si>
+    <t>Casque ACH (Advanced Combat Helmet)</t>
+  </si>
+  <si>
+    <t>Casque FAST Ballistic</t>
+  </si>
+  <si>
+    <t>Casque lourd EOD</t>
+  </si>
+  <si>
+    <t>Armures\Membres</t>
+  </si>
+  <si>
+    <t>Brassards de protection</t>
+  </si>
+  <si>
+    <t>Kit protection membres complet</t>
+  </si>
+  <si>
+    <t>Armures\Completes</t>
+  </si>
+  <si>
+    <t>Equipement\Medical</t>
+  </si>
+  <si>
+    <t>Trousse de premiers secours légère</t>
+  </si>
+  <si>
+    <t>Bandages stériles, désinfectant, garrot CAT — traitement blessures légères</t>
+  </si>
+  <si>
+    <t>Kit de trauma tactique (IFAK)</t>
+  </si>
+  <si>
+    <t>Pansement hémostatique QuikClot, décompression thoracique, garrot CAT, gants nitrile</t>
+  </si>
+  <si>
+    <t>Trousse médicale avancée (TCCC)</t>
+  </si>
+  <si>
+    <t>Matériel réanimation, intubation nasopharyngée, sutures, traitement multi-plaies graves</t>
+  </si>
+  <si>
+    <t>Défibrillateur portable DEA</t>
+  </si>
+  <si>
+    <t>Défibrillateur automatique externe — usage par personnel non médical</t>
+  </si>
+  <si>
+    <t>Auto-injecteur morphine x5</t>
+  </si>
+  <si>
+    <t>5 auto-injecteurs morphine 10mg — analgésie d'urgence au combat</t>
+  </si>
+  <si>
+    <t>Garrot tourniquet CAT x3</t>
+  </si>
+  <si>
+    <t>3 garrots Combat Application Tourniquet — 1 main possible — norme TCCC</t>
+  </si>
+  <si>
+    <t>Equipement\Communication</t>
+  </si>
+  <si>
+    <t>Radio MBITR AN/PRC-148</t>
+  </si>
+  <si>
+    <t>Radio militaire multi-bandes sécurisée — portée 5km sol-sol avec chiffrement</t>
+  </si>
+  <si>
+    <t>Radio longue portée AN/PRC-117G</t>
+  </si>
+  <si>
+    <t>Radio tactique wideband avec capacité satcom — portée 50km+</t>
+  </si>
+  <si>
+    <t>Casque tactique Peltor ComTac IV</t>
+  </si>
+  <si>
+    <t>Protection auditive active avec passerelle radio intégrée — atténuation 26dB</t>
+  </si>
+  <si>
+    <t>Balise de détresse PLB 406MHz</t>
+  </si>
+  <si>
+    <t>Balise localisatrice personnelle COSPAS-SARSAT — activation manuelle ou automatique</t>
+  </si>
+  <si>
+    <t>Système de communication intra-équipe</t>
+  </si>
+  <si>
+    <t>Kit PTT discret avec écouteur intra et micro laryngophone — discrétion opérationnelle</t>
+  </si>
+  <si>
+    <t>Equipement\Optique</t>
+  </si>
+  <si>
+    <t>Jumelles 8x42 tactiques</t>
+  </si>
+  <si>
+    <t>Jumelles milspecs résistantes chocs et eau — champ de vision 130m/1000m</t>
+  </si>
+  <si>
+    <t>Monoculaire NV AN/PVS-14 Gen III</t>
+  </si>
+  <si>
+    <t>Intensificateur de lumière Gen III — vision nocturne opérationnelle 0 à 300m</t>
+  </si>
+  <si>
+    <t>Caméra thermique FLIR Scout III</t>
+  </si>
+  <si>
+    <t>Analyse thermique IR longue portée — détection silhouettes humaines à 500m+</t>
+  </si>
+  <si>
+    <t>Télémètre laser Vectronix PLRF</t>
+  </si>
+  <si>
+    <t>Télémètre militaire 25m-10km avec boussole numérique et GPS intégré</t>
+  </si>
+  <si>
+    <t>Equipement\CBRN</t>
+  </si>
+  <si>
+    <t>Masque respiratoire M50</t>
+  </si>
+  <si>
+    <t>Masque gaz militaire — protection agents chimiques et biologiques — autonomie 24h</t>
+  </si>
+  <si>
+    <t>Détecteur d'agents chimiques M8A1</t>
+  </si>
+  <si>
+    <t>Détecteur automatique agents neurotoxiques et vésicants — alarme sonore et visuelle</t>
+  </si>
+  <si>
+    <t>Tenue MOPP4 complète</t>
+  </si>
+  <si>
+    <t>Ensemble protecteur NBC intégral (masque non inclus) — résistance certifiée 24h</t>
+  </si>
+  <si>
+    <t>Tablettes décontamination RSDL x10</t>
+  </si>
+  <si>
+    <t>10 lingettes décontaminantes peau — neutralisation agents chimiques en 2min</t>
+  </si>
+  <si>
+    <t>Equipement\Transport</t>
+  </si>
+  <si>
+    <t>Sac d'assaut MOLLE 45L</t>
+  </si>
+  <si>
+    <t>Sac à dos tactique modulaire MOLLE — tissu 1000D Cordura — capacité 45L</t>
+  </si>
+  <si>
+    <t>Porte-plaques tactique (PC) MOLLE</t>
+  </si>
+  <si>
+    <t>Porte-équipement MOLLE sans plaques — transport matériel combat 15 poches modulaires</t>
+  </si>
+  <si>
+    <t>Ceinturon ALICE avec accessoires</t>
+  </si>
+  <si>
+    <t>Ceinturon militaire avec porte-gourde, poches munitions et holster toile</t>
+  </si>
+  <si>
+    <t>Caisse de transport Pelican 1510</t>
+  </si>
+  <si>
+    <t>Malette rigide étanche IP67 — transport équipement sensible 56x36x23cm</t>
+  </si>
+  <si>
+    <t>Equipement\Survie</t>
+  </si>
+  <si>
+    <t>Kit de survie 72h</t>
+  </si>
+  <si>
+    <t>Eau purifiée, barres énergétiques, bivouac urgence, allumettes tempête, miroir signal</t>
+  </si>
+  <si>
+    <t>Couvertures thermiques de survie x3</t>
+  </si>
+  <si>
+    <t>Couvertures aluminisées réfléchissantes — protection hypothermie jusqu'à -20°C</t>
+  </si>
+  <si>
+    <t>Filtre à eau LifeStraw Mission</t>
+  </si>
+  <si>
+    <t>Filtre portatif 1L/min — élimination 99,9999% bactéries et 99,9% parasites</t>
+  </si>
+  <si>
+    <t>GPS militaire Garmin GPSMAP 64sx</t>
+  </si>
+  <si>
+    <t>GPS milspecs IP68 — cartes topo MGRS — autonomie 16h batteries AA</t>
+  </si>
+  <si>
+    <t>Equipement\Eclairage</t>
+  </si>
+  <si>
+    <t>Lampe tactique Streamlight TLR-1</t>
+  </si>
+  <si>
+    <t>Lampe rail Picatinny 300 lumens — activation ambidextre — IP54</t>
+  </si>
+  <si>
+    <t>Lampe frontale militaire THL-1 NV</t>
+  </si>
+  <si>
+    <t>Lampe frontale 4 modes: blanc/rouge/IR/strobe — compatible NVG</t>
+  </si>
+  <si>
+    <t>Bâtons lumineux chimiques x10</t>
+  </si>
+  <si>
+    <t>Cyalume 12h — balisage et jalonnement discret — spectre vert et infrarouge</t>
+  </si>
+  <si>
+    <t>Equipement\Outils</t>
+  </si>
+  <si>
+    <t>Outil multifonction Leatherman MUT</t>
+  </si>
+  <si>
+    <t>Outil multifonction avec adaptateur nettoyage arme, chasse-goupille et kit AR</t>
+  </si>
+  <si>
+    <t>Pince coupe-barbelés renforcée</t>
+  </si>
+  <si>
+    <t>Pince coupe acier galvanisé 5mm et câble acier 3mm — manche isolé</t>
+  </si>
+  <si>
+    <t>Pied de biche tactique compact</t>
+  </si>
+  <si>
+    <t>Pied de biche acier forgé 35cm — forçage portes et extraction matériel</t>
+  </si>
+  <si>
+    <t>Scie-câble de survie</t>
+  </si>
+  <si>
+    <t>Scie-câble acier inox — coupe bois, os et matériaux composites légers</t>
+  </si>
+  <si>
+    <t>Détecteur de métaux Garrett THD</t>
+  </si>
+  <si>
+    <t>Détecteur de métaux portable — mines PT et IED à moins de 15cm — mode discrimination</t>
+  </si>
+  <si>
+    <t>Protection balistique légère contre petits calibres — arrête les fragments et chevrotines</t>
+  </si>
+  <si>
+    <t>Protection contre munitions FMJ 9mm et .40 S&amp;W basse vélocité</t>
+  </si>
+  <si>
+    <t>Protection contre munitions FMJ .357 Magnum et 9mm haute vélocité</t>
+  </si>
+  <si>
+    <t>Protection contre munitions .44 Magnum et SMG — port discret possible</t>
+  </si>
+  <si>
+    <t>Gilet NIJ IIIA avec rehausse cervicale — protection poitrine, abdomen, bas-ventre et cou</t>
+  </si>
+  <si>
+    <t>Gilet opérationnel avec poches plaques avant/arrière ESAPI NIJ IV + panneaux latéraux</t>
+  </si>
+  <si>
+    <t>Armure composite disc-céramique révolutionnaire — haute résistance sur toute la zone tronc</t>
+  </si>
+  <si>
+    <t>Tenue NBC avec gilet anti-fragmentation intégré — protection chimique 8h</t>
+  </si>
+  <si>
+    <t>Tenue EOD légère</t>
+  </si>
+  <si>
+    <t>Protection contre explosions et fragmentation pour opérations déminage légères</t>
+  </si>
+  <si>
+    <t>Casque kevlar utilisé par les forces armées américaines depuis 1983 — protection balistique sol</t>
+  </si>
+  <si>
+    <t>Casque modulaire rails latéraux — compatible NVG, caméra et systèmes de communication</t>
+  </si>
+  <si>
+    <t>Casque allégé coupe haute — compatibilité systèmes de communication et interphone</t>
+  </si>
+  <si>
+    <t>Casque Galvion Caiman avec visière</t>
+  </si>
+  <si>
+    <t>Casque balistique haut de gamme avec visière balistique NIJ IIIA escamotable</t>
+  </si>
+  <si>
+    <t>Casque intégral demi-sphère pour opérations déminage — protection visage et cou</t>
+  </si>
+  <si>
+    <t>Coudières tactiques Hatch</t>
+  </si>
+  <si>
+    <t>Protection polymère renforcée pour coudes — compatibles sous-vêtement ou sur uniforme</t>
+  </si>
+  <si>
+    <t>Genouillères tactiques Hatch</t>
+  </si>
+  <si>
+    <t>Genouillères à glissière gel anatomique — positions de tir prolongées</t>
+  </si>
+  <si>
+    <t>Protection avant-bras contre éclats et contusions en milieu urbain</t>
+  </si>
+  <si>
+    <t>Jambières tactiques balistiques</t>
+  </si>
+  <si>
+    <t>Protection jambe basse et cheville — milieu urbain et opérations de brèche</t>
+  </si>
+  <si>
+    <t>Ensemble brassards + genouillères + coudières — protection périphérique complète</t>
+  </si>
+  <si>
+    <t>Armure légère complète (LAW)</t>
+  </si>
+  <si>
+    <t>Casque ACH + gilet NIJ IIIA + protection membres légère — configuration d'intervention</t>
+  </si>
+  <si>
+    <t>Armure assault complète (SAP)</t>
+  </si>
+  <si>
+    <t>IOTV + casque FAST + membres — configuration assaut haute intensité</t>
+  </si>
+  <si>
+    <t>Exosquelette de combat léger</t>
+  </si>
+  <si>
+    <t>Exosquelette balistique assisté motorisé — protection renforcée toutes zones</t>
   </si>
 </sst>
 </file>
@@ -2811,7 +3417,7 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -2902,6 +3508,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="6"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Accent1" xfId="3" builtinId="29"/>
@@ -49718,7 +50325,7 @@
         <v>832</v>
       </c>
       <c r="U322" s="28">
-        <f t="shared" ref="U322:U385" si="62">T322 * POWER(I322/S322,0.25)</f>
+        <f t="shared" ref="U322:U383" si="62">T322 * POWER(I322/S322,0.25)</f>
         <v>768.32975389098669</v>
       </c>
       <c r="V322" s="26">
@@ -57341,6 +57948,3727 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41A94B5E-6234-47BA-BD31-8138FCAAF115}">
+  <dimension ref="A1:N30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="14" max="14" width="48.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="B1" t="s">
+        <v>868</v>
+      </c>
+      <c r="C1" t="s">
+        <v>916</v>
+      </c>
+      <c r="D1" t="s">
+        <v>869</v>
+      </c>
+      <c r="E1" t="s">
+        <v>917</v>
+      </c>
+      <c r="F1" t="s">
+        <v>918</v>
+      </c>
+      <c r="G1" t="s">
+        <v>919</v>
+      </c>
+      <c r="H1" t="s">
+        <v>870</v>
+      </c>
+      <c r="I1" t="s">
+        <v>871</v>
+      </c>
+      <c r="J1" t="s">
+        <v>872</v>
+      </c>
+      <c r="K1" t="s">
+        <v>873</v>
+      </c>
+      <c r="L1" t="s">
+        <v>874</v>
+      </c>
+      <c r="M1" t="s">
+        <v>875</v>
+      </c>
+      <c r="N1" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="str">
+        <f>_xlfn.CONCAT("Feature\" &amp; B2)</f>
+        <v>Feature\Visée rudimentaire</v>
+      </c>
+      <c r="B2" t="s">
+        <v>877</v>
+      </c>
+      <c r="C2" t="s">
+        <v>878</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="str">
+        <f t="shared" ref="A3:A30" si="0">_xlfn.CONCAT("Feature\" &amp; B3)</f>
+        <v>Feature\Visée rudimentaire</v>
+      </c>
+      <c r="B3" t="s">
+        <v>877</v>
+      </c>
+      <c r="C3" t="s">
+        <v>879</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée rudimentaire</v>
+      </c>
+      <c r="B4" t="s">
+        <v>877</v>
+      </c>
+      <c r="C4" t="s">
+        <v>880</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée rudimentaire</v>
+      </c>
+      <c r="B5" t="s">
+        <v>877</v>
+      </c>
+      <c r="C5" t="s">
+        <v>881</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0.17499999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B6" t="s">
+        <v>882</v>
+      </c>
+      <c r="C6" t="s">
+        <v>883</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B7" t="s">
+        <v>882</v>
+      </c>
+      <c r="C7" t="s">
+        <v>884</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B8" t="s">
+        <v>882</v>
+      </c>
+      <c r="C8" t="s">
+        <v>885</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B9" t="s">
+        <v>882</v>
+      </c>
+      <c r="C9" t="s">
+        <v>886</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B10" t="s">
+        <v>882</v>
+      </c>
+      <c r="C10" t="s">
+        <v>887</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B11" t="s">
+        <v>882</v>
+      </c>
+      <c r="C11" t="s">
+        <v>888</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B12" t="s">
+        <v>882</v>
+      </c>
+      <c r="C12" t="s">
+        <v>889</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>3</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B13" t="s">
+        <v>882</v>
+      </c>
+      <c r="C13" t="s">
+        <v>890</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0.52500000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B14" t="s">
+        <v>882</v>
+      </c>
+      <c r="C14" t="s">
+        <v>891</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B15" t="s">
+        <v>882</v>
+      </c>
+      <c r="C15" t="s">
+        <v>892</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B16" t="s">
+        <v>882</v>
+      </c>
+      <c r="C16" t="s">
+        <v>893</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16">
+        <v>2</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B17" t="s">
+        <v>882</v>
+      </c>
+      <c r="C17" t="s">
+        <v>894</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B18" t="s">
+        <v>882</v>
+      </c>
+      <c r="C18" t="s">
+        <v>895</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>2</v>
+      </c>
+      <c r="G18">
+        <v>3</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B19" t="s">
+        <v>882</v>
+      </c>
+      <c r="C19" t="s">
+        <v>896</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B20" t="s">
+        <v>882</v>
+      </c>
+      <c r="C20" t="s">
+        <v>897</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>0.42499999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Visée lunette</v>
+      </c>
+      <c r="B21" t="s">
+        <v>882</v>
+      </c>
+      <c r="C21" t="s">
+        <v>898</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Addons</v>
+      </c>
+      <c r="B22" t="s">
+        <v>899</v>
+      </c>
+      <c r="C22" t="s">
+        <v>900</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>0.1</v>
+      </c>
+      <c r="N22" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Addons</v>
+      </c>
+      <c r="B23" t="s">
+        <v>899</v>
+      </c>
+      <c r="C23" t="s">
+        <v>902</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
+      <c r="A24" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Silencieux</v>
+      </c>
+      <c r="B24" t="s">
+        <v>903</v>
+      </c>
+      <c r="C24" t="s">
+        <v>904</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24" s="36">
+        <v>-0.8</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Silencieux</v>
+      </c>
+      <c r="B25" t="s">
+        <v>903</v>
+      </c>
+      <c r="C25" t="s">
+        <v>905</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>-25</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>17.5</v>
+      </c>
+      <c r="M25">
+        <v>0.3</v>
+      </c>
+      <c r="N25" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Silencieux</v>
+      </c>
+      <c r="B26" t="s">
+        <v>903</v>
+      </c>
+      <c r="C26" t="s">
+        <v>907</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>-35</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>13</v>
+      </c>
+      <c r="M26">
+        <v>0.1</v>
+      </c>
+      <c r="N26" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
+      <c r="A27" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Silencieux</v>
+      </c>
+      <c r="B27" t="s">
+        <v>903</v>
+      </c>
+      <c r="C27" t="s">
+        <v>909</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>-55</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>32.5</v>
+      </c>
+      <c r="M27">
+        <v>0.8</v>
+      </c>
+      <c r="N27" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
+      <c r="A28" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Silencieux</v>
+      </c>
+      <c r="B28" t="s">
+        <v>903</v>
+      </c>
+      <c r="C28" t="s">
+        <v>911</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>-40</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>17.5</v>
+      </c>
+      <c r="M28">
+        <v>0.2</v>
+      </c>
+      <c r="N28" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="A29" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Silencieux</v>
+      </c>
+      <c r="B29" t="s">
+        <v>903</v>
+      </c>
+      <c r="C29" t="s">
+        <v>912</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>-50</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>30</v>
+      </c>
+      <c r="M29">
+        <v>0.6</v>
+      </c>
+      <c r="N29" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
+      <c r="A30" t="str">
+        <f t="shared" si="0"/>
+        <v>Feature\Silencieux</v>
+      </c>
+      <c r="B30" t="s">
+        <v>903</v>
+      </c>
+      <c r="C30" t="s">
+        <v>914</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>-70</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>42.5</v>
+      </c>
+      <c r="M30">
+        <v>1.2</v>
+      </c>
+      <c r="N30" t="s">
+        <v>915</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81B44A9-9026-4248-B1DC-F446852477BC}">
+  <dimension ref="A1:Z23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="94" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26">
+      <c r="A1" t="s">
+        <v>575</v>
+      </c>
+      <c r="B1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" t="s">
+        <v>873</v>
+      </c>
+      <c r="D1" t="s">
+        <v>874</v>
+      </c>
+      <c r="E1" t="s">
+        <v>875</v>
+      </c>
+      <c r="F1" t="s">
+        <v>876</v>
+      </c>
+      <c r="G1" t="s">
+        <v>920</v>
+      </c>
+      <c r="H1" t="s">
+        <v>921</v>
+      </c>
+      <c r="I1" t="s">
+        <v>922</v>
+      </c>
+      <c r="J1" t="s">
+        <v>923</v>
+      </c>
+      <c r="K1" t="s">
+        <v>924</v>
+      </c>
+      <c r="L1" t="s">
+        <v>925</v>
+      </c>
+      <c r="M1" t="s">
+        <v>926</v>
+      </c>
+      <c r="N1" t="s">
+        <v>927</v>
+      </c>
+      <c r="O1" t="s">
+        <v>928</v>
+      </c>
+      <c r="P1" t="s">
+        <v>929</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>930</v>
+      </c>
+      <c r="R1" t="s">
+        <v>931</v>
+      </c>
+      <c r="S1" t="s">
+        <v>932</v>
+      </c>
+      <c r="T1" t="s">
+        <v>933</v>
+      </c>
+      <c r="U1" t="s">
+        <v>934</v>
+      </c>
+      <c r="V1" t="s">
+        <v>935</v>
+      </c>
+      <c r="W1" t="s">
+        <v>936</v>
+      </c>
+      <c r="X1" t="s">
+        <v>937</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>938</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26">
+      <c r="A2" t="s">
+        <v>940</v>
+      </c>
+      <c r="B2" t="s">
+        <v>941</v>
+      </c>
+      <c r="C2" t="s">
+        <v>942</v>
+      </c>
+      <c r="D2">
+        <v>200</v>
+      </c>
+      <c r="E2">
+        <v>1.2</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1039</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26">
+      <c r="A3" t="s">
+        <v>940</v>
+      </c>
+      <c r="B3" t="s">
+        <v>943</v>
+      </c>
+      <c r="C3" t="s">
+        <v>942</v>
+      </c>
+      <c r="D3">
+        <v>350</v>
+      </c>
+      <c r="E3">
+        <v>1.8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1040</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+      <c r="N3">
+        <v>2</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26">
+      <c r="A4" t="s">
+        <v>940</v>
+      </c>
+      <c r="B4" t="s">
+        <v>944</v>
+      </c>
+      <c r="C4" t="s">
+        <v>942</v>
+      </c>
+      <c r="D4">
+        <v>500</v>
+      </c>
+      <c r="E4">
+        <v>2.5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1041</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
+      </c>
+      <c r="N4">
+        <v>3</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26">
+      <c r="A5" t="s">
+        <v>940</v>
+      </c>
+      <c r="B5" t="s">
+        <v>945</v>
+      </c>
+      <c r="C5" t="s">
+        <v>946</v>
+      </c>
+      <c r="D5">
+        <v>800</v>
+      </c>
+      <c r="E5">
+        <v>3.2</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1042</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>4</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
+      <c r="N5">
+        <v>4</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+      <c r="Z5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26">
+      <c r="A6" t="s">
+        <v>940</v>
+      </c>
+      <c r="B6" t="s">
+        <v>947</v>
+      </c>
+      <c r="C6" t="s">
+        <v>946</v>
+      </c>
+      <c r="D6">
+        <v>1100</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1043</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>4</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+      <c r="N6">
+        <v>4</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26">
+      <c r="A7" t="s">
+        <v>940</v>
+      </c>
+      <c r="B7" t="s">
+        <v>948</v>
+      </c>
+      <c r="C7" t="s">
+        <v>946</v>
+      </c>
+      <c r="D7">
+        <v>2200</v>
+      </c>
+      <c r="E7">
+        <v>7.5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1044</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>8</v>
+      </c>
+      <c r="K7">
+        <v>8</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>7</v>
+      </c>
+      <c r="N7">
+        <v>6</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26">
+      <c r="A8" t="s">
+        <v>940</v>
+      </c>
+      <c r="B8" t="s">
+        <v>949</v>
+      </c>
+      <c r="C8" t="s">
+        <v>950</v>
+      </c>
+      <c r="D8">
+        <v>6500</v>
+      </c>
+      <c r="E8">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1045</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8">
+        <v>10</v>
+      </c>
+      <c r="K8">
+        <v>10</v>
+      </c>
+      <c r="L8">
+        <v>9</v>
+      </c>
+      <c r="M8">
+        <v>9</v>
+      </c>
+      <c r="N8">
+        <v>8</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26">
+      <c r="A9" t="s">
+        <v>940</v>
+      </c>
+      <c r="B9" t="s">
+        <v>951</v>
+      </c>
+      <c r="C9" t="s">
+        <v>950</v>
+      </c>
+      <c r="D9">
+        <v>4500</v>
+      </c>
+      <c r="E9">
+        <v>5.8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1046</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>2</v>
+      </c>
+      <c r="J9">
+        <v>5</v>
+      </c>
+      <c r="K9">
+        <v>5</v>
+      </c>
+      <c r="L9">
+        <v>5</v>
+      </c>
+      <c r="M9">
+        <v>5</v>
+      </c>
+      <c r="N9">
+        <v>5</v>
+      </c>
+      <c r="O9">
+        <v>2</v>
+      </c>
+      <c r="P9">
+        <v>2</v>
+      </c>
+      <c r="Q9">
+        <v>2</v>
+      </c>
+      <c r="R9">
+        <v>2</v>
+      </c>
+      <c r="S9">
+        <v>1</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="U9">
+        <v>2</v>
+      </c>
+      <c r="V9">
+        <v>2</v>
+      </c>
+      <c r="W9">
+        <v>2</v>
+      </c>
+      <c r="X9">
+        <v>2</v>
+      </c>
+      <c r="Y9">
+        <v>1</v>
+      </c>
+      <c r="Z9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26">
+      <c r="A10" t="s">
+        <v>940</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C10" t="s">
+        <v>950</v>
+      </c>
+      <c r="D10">
+        <v>12000</v>
+      </c>
+      <c r="E10">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1048</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>3</v>
+      </c>
+      <c r="J10">
+        <v>7</v>
+      </c>
+      <c r="K10">
+        <v>7</v>
+      </c>
+      <c r="L10">
+        <v>7</v>
+      </c>
+      <c r="M10">
+        <v>7</v>
+      </c>
+      <c r="N10">
+        <v>7</v>
+      </c>
+      <c r="O10">
+        <v>3</v>
+      </c>
+      <c r="P10">
+        <v>3</v>
+      </c>
+      <c r="Q10">
+        <v>3</v>
+      </c>
+      <c r="R10">
+        <v>3</v>
+      </c>
+      <c r="S10">
+        <v>2</v>
+      </c>
+      <c r="T10">
+        <v>2</v>
+      </c>
+      <c r="U10">
+        <v>3</v>
+      </c>
+      <c r="V10">
+        <v>3</v>
+      </c>
+      <c r="W10">
+        <v>3</v>
+      </c>
+      <c r="X10">
+        <v>3</v>
+      </c>
+      <c r="Y10">
+        <v>2</v>
+      </c>
+      <c r="Z10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26">
+      <c r="A11" t="s">
+        <v>952</v>
+      </c>
+      <c r="B11" t="s">
+        <v>953</v>
+      </c>
+      <c r="C11" t="s">
+        <v>942</v>
+      </c>
+      <c r="D11">
+        <v>180</v>
+      </c>
+      <c r="E11">
+        <v>1.4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>1049</v>
+      </c>
+      <c r="G11">
+        <v>3</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26">
+      <c r="A12" t="s">
+        <v>952</v>
+      </c>
+      <c r="B12" t="s">
+        <v>954</v>
+      </c>
+      <c r="C12" t="s">
+        <v>942</v>
+      </c>
+      <c r="D12">
+        <v>380</v>
+      </c>
+      <c r="E12">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F12" t="s">
+        <v>1050</v>
+      </c>
+      <c r="G12">
+        <v>4</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>0</v>
+      </c>
+      <c r="Y12">
+        <v>0</v>
+      </c>
+      <c r="Z12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26">
+      <c r="A13" t="s">
+        <v>952</v>
+      </c>
+      <c r="B13" t="s">
+        <v>955</v>
+      </c>
+      <c r="C13" t="s">
+        <v>946</v>
+      </c>
+      <c r="D13">
+        <v>620</v>
+      </c>
+      <c r="E13">
+        <v>0.9</v>
+      </c>
+      <c r="F13" t="s">
+        <v>1051</v>
+      </c>
+      <c r="G13">
+        <v>4</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>0</v>
+      </c>
+      <c r="Y13">
+        <v>0</v>
+      </c>
+      <c r="Z13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26">
+      <c r="A14" t="s">
+        <v>952</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C14" t="s">
+        <v>950</v>
+      </c>
+      <c r="D14">
+        <v>1800</v>
+      </c>
+      <c r="E14">
+        <v>1.3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G14">
+        <v>4</v>
+      </c>
+      <c r="H14">
+        <v>3</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26">
+      <c r="A15" t="s">
+        <v>952</v>
+      </c>
+      <c r="B15" t="s">
+        <v>956</v>
+      </c>
+      <c r="C15" t="s">
+        <v>950</v>
+      </c>
+      <c r="D15">
+        <v>3200</v>
+      </c>
+      <c r="E15">
+        <v>3.5</v>
+      </c>
+      <c r="F15" t="s">
+        <v>1054</v>
+      </c>
+      <c r="G15">
+        <v>5</v>
+      </c>
+      <c r="H15">
+        <v>4</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
+        <v>0</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26">
+      <c r="A16" t="s">
+        <v>957</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C16" t="s">
+        <v>942</v>
+      </c>
+      <c r="D16">
+        <v>80</v>
+      </c>
+      <c r="E16">
+        <v>0.6</v>
+      </c>
+      <c r="F16" t="s">
+        <v>1056</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>2</v>
+      </c>
+      <c r="R16">
+        <v>2</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <v>0</v>
+      </c>
+      <c r="V16">
+        <v>0</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>0</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26">
+      <c r="A17" t="s">
+        <v>957</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C17" t="s">
+        <v>942</v>
+      </c>
+      <c r="D17">
+        <v>90</v>
+      </c>
+      <c r="E17">
+        <v>0.7</v>
+      </c>
+      <c r="F17" t="s">
+        <v>1058</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <v>0</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>2</v>
+      </c>
+      <c r="X17">
+        <v>2</v>
+      </c>
+      <c r="Y17">
+        <v>0</v>
+      </c>
+      <c r="Z17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26">
+      <c r="A18" t="s">
+        <v>957</v>
+      </c>
+      <c r="B18" t="s">
+        <v>958</v>
+      </c>
+      <c r="C18" t="s">
+        <v>942</v>
+      </c>
+      <c r="D18">
+        <v>120</v>
+      </c>
+      <c r="E18">
+        <v>0.8</v>
+      </c>
+      <c r="F18" t="s">
+        <v>1059</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>2</v>
+      </c>
+      <c r="P18">
+        <v>2</v>
+      </c>
+      <c r="Q18">
+        <v>2</v>
+      </c>
+      <c r="R18">
+        <v>2</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <v>0</v>
+      </c>
+      <c r="V18">
+        <v>0</v>
+      </c>
+      <c r="W18">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>0</v>
+      </c>
+      <c r="Y18">
+        <v>0</v>
+      </c>
+      <c r="Z18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26">
+      <c r="A19" t="s">
+        <v>957</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1060</v>
+      </c>
+      <c r="C19" t="s">
+        <v>942</v>
+      </c>
+      <c r="D19">
+        <v>150</v>
+      </c>
+      <c r="E19">
+        <v>1.4</v>
+      </c>
+      <c r="F19" t="s">
+        <v>1061</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <v>0</v>
+      </c>
+      <c r="V19">
+        <v>0</v>
+      </c>
+      <c r="W19">
+        <v>2</v>
+      </c>
+      <c r="X19">
+        <v>2</v>
+      </c>
+      <c r="Y19">
+        <v>2</v>
+      </c>
+      <c r="Z19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26">
+      <c r="A20" t="s">
+        <v>957</v>
+      </c>
+      <c r="B20" t="s">
+        <v>959</v>
+      </c>
+      <c r="C20" t="s">
+        <v>946</v>
+      </c>
+      <c r="D20">
+        <v>450</v>
+      </c>
+      <c r="E20">
+        <v>3.5</v>
+      </c>
+      <c r="F20" t="s">
+        <v>1062</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>2</v>
+      </c>
+      <c r="P20">
+        <v>2</v>
+      </c>
+      <c r="Q20">
+        <v>3</v>
+      </c>
+      <c r="R20">
+        <v>3</v>
+      </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>0</v>
+      </c>
+      <c r="U20">
+        <v>0</v>
+      </c>
+      <c r="V20">
+        <v>0</v>
+      </c>
+      <c r="W20">
+        <v>3</v>
+      </c>
+      <c r="X20">
+        <v>3</v>
+      </c>
+      <c r="Y20">
+        <v>2</v>
+      </c>
+      <c r="Z20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:26">
+      <c r="A21" t="s">
+        <v>960</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C21" t="s">
+        <v>946</v>
+      </c>
+      <c r="D21">
+        <v>3500</v>
+      </c>
+      <c r="E21">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1064</v>
+      </c>
+      <c r="G21">
+        <v>3</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <v>4</v>
+      </c>
+      <c r="K21">
+        <v>4</v>
+      </c>
+      <c r="L21">
+        <v>4</v>
+      </c>
+      <c r="M21">
+        <v>4</v>
+      </c>
+      <c r="N21">
+        <v>4</v>
+      </c>
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21">
+        <v>1</v>
+      </c>
+      <c r="Q21">
+        <v>2</v>
+      </c>
+      <c r="R21">
+        <v>2</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
+      <c r="U21">
+        <v>1</v>
+      </c>
+      <c r="V21">
+        <v>1</v>
+      </c>
+      <c r="W21">
+        <v>2</v>
+      </c>
+      <c r="X21">
+        <v>2</v>
+      </c>
+      <c r="Y21">
+        <v>1</v>
+      </c>
+      <c r="Z21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26">
+      <c r="A22" t="s">
+        <v>960</v>
+      </c>
+      <c r="B22" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C22" t="s">
+        <v>950</v>
+      </c>
+      <c r="D22">
+        <v>8500</v>
+      </c>
+      <c r="E22">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>1066</v>
+      </c>
+      <c r="G22">
+        <v>4</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
+      <c r="J22">
+        <v>8</v>
+      </c>
+      <c r="K22">
+        <v>8</v>
+      </c>
+      <c r="L22">
+        <v>7</v>
+      </c>
+      <c r="M22">
+        <v>7</v>
+      </c>
+      <c r="N22">
+        <v>6</v>
+      </c>
+      <c r="O22">
+        <v>2</v>
+      </c>
+      <c r="P22">
+        <v>2</v>
+      </c>
+      <c r="Q22">
+        <v>3</v>
+      </c>
+      <c r="R22">
+        <v>3</v>
+      </c>
+      <c r="S22">
+        <v>1</v>
+      </c>
+      <c r="T22">
+        <v>1</v>
+      </c>
+      <c r="U22">
+        <v>2</v>
+      </c>
+      <c r="V22">
+        <v>2</v>
+      </c>
+      <c r="W22">
+        <v>3</v>
+      </c>
+      <c r="X22">
+        <v>3</v>
+      </c>
+      <c r="Y22">
+        <v>2</v>
+      </c>
+      <c r="Z22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:26">
+      <c r="A23" t="s">
+        <v>960</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C23" t="s">
+        <v>950</v>
+      </c>
+      <c r="D23">
+        <v>45000</v>
+      </c>
+      <c r="E23">
+        <v>15</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G23">
+        <v>3</v>
+      </c>
+      <c r="H23">
+        <v>2</v>
+      </c>
+      <c r="I23">
+        <v>2</v>
+      </c>
+      <c r="J23">
+        <v>6</v>
+      </c>
+      <c r="K23">
+        <v>6</v>
+      </c>
+      <c r="L23">
+        <v>5</v>
+      </c>
+      <c r="M23">
+        <v>5</v>
+      </c>
+      <c r="N23">
+        <v>5</v>
+      </c>
+      <c r="O23">
+        <v>4</v>
+      </c>
+      <c r="P23">
+        <v>4</v>
+      </c>
+      <c r="Q23">
+        <v>4</v>
+      </c>
+      <c r="R23">
+        <v>4</v>
+      </c>
+      <c r="S23">
+        <v>2</v>
+      </c>
+      <c r="T23">
+        <v>2</v>
+      </c>
+      <c r="U23">
+        <v>4</v>
+      </c>
+      <c r="V23">
+        <v>4</v>
+      </c>
+      <c r="W23">
+        <v>4</v>
+      </c>
+      <c r="X23">
+        <v>4</v>
+      </c>
+      <c r="Y23">
+        <v>3</v>
+      </c>
+      <c r="Z23">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30045938-0EF7-4DB0-8EC0-CD7790E40548}">
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="83.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>575</v>
+      </c>
+      <c r="B1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" t="s">
+        <v>873</v>
+      </c>
+      <c r="D1" t="s">
+        <v>874</v>
+      </c>
+      <c r="E1" t="s">
+        <v>875</v>
+      </c>
+      <c r="F1" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>961</v>
+      </c>
+      <c r="B2" t="s">
+        <v>962</v>
+      </c>
+      <c r="C2" t="s">
+        <v>942</v>
+      </c>
+      <c r="D2">
+        <v>50</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>961</v>
+      </c>
+      <c r="B3" t="s">
+        <v>964</v>
+      </c>
+      <c r="C3" t="s">
+        <v>942</v>
+      </c>
+      <c r="D3">
+        <v>200</v>
+      </c>
+      <c r="E3">
+        <v>0.8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>961</v>
+      </c>
+      <c r="B4" t="s">
+        <v>966</v>
+      </c>
+      <c r="C4" t="s">
+        <v>946</v>
+      </c>
+      <c r="D4">
+        <v>600</v>
+      </c>
+      <c r="E4">
+        <v>3.5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>961</v>
+      </c>
+      <c r="B5" t="s">
+        <v>968</v>
+      </c>
+      <c r="C5" t="s">
+        <v>946</v>
+      </c>
+      <c r="D5">
+        <v>1200</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>961</v>
+      </c>
+      <c r="B6" t="s">
+        <v>970</v>
+      </c>
+      <c r="C6" t="s">
+        <v>946</v>
+      </c>
+      <c r="D6">
+        <v>150</v>
+      </c>
+      <c r="E6">
+        <v>0.1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>961</v>
+      </c>
+      <c r="B7" t="s">
+        <v>972</v>
+      </c>
+      <c r="C7" t="s">
+        <v>942</v>
+      </c>
+      <c r="D7">
+        <v>45</v>
+      </c>
+      <c r="E7">
+        <v>0.1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>974</v>
+      </c>
+      <c r="B8" t="s">
+        <v>975</v>
+      </c>
+      <c r="C8" t="s">
+        <v>946</v>
+      </c>
+      <c r="D8">
+        <v>3500</v>
+      </c>
+      <c r="E8">
+        <v>0.6</v>
+      </c>
+      <c r="F8" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>974</v>
+      </c>
+      <c r="B9" t="s">
+        <v>977</v>
+      </c>
+      <c r="C9" t="s">
+        <v>950</v>
+      </c>
+      <c r="D9">
+        <v>8000</v>
+      </c>
+      <c r="E9">
+        <v>5</v>
+      </c>
+      <c r="F9" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>974</v>
+      </c>
+      <c r="B10" t="s">
+        <v>979</v>
+      </c>
+      <c r="C10" t="s">
+        <v>942</v>
+      </c>
+      <c r="D10">
+        <v>800</v>
+      </c>
+      <c r="E10">
+        <v>0.4</v>
+      </c>
+      <c r="F10" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>974</v>
+      </c>
+      <c r="B11" t="s">
+        <v>981</v>
+      </c>
+      <c r="C11" t="s">
+        <v>942</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11">
+        <v>0.2</v>
+      </c>
+      <c r="F11" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>974</v>
+      </c>
+      <c r="B12" t="s">
+        <v>983</v>
+      </c>
+      <c r="C12" t="s">
+        <v>946</v>
+      </c>
+      <c r="D12">
+        <v>1200</v>
+      </c>
+      <c r="E12">
+        <v>0.3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>985</v>
+      </c>
+      <c r="B13" t="s">
+        <v>986</v>
+      </c>
+      <c r="C13" t="s">
+        <v>942</v>
+      </c>
+      <c r="D13">
+        <v>200</v>
+      </c>
+      <c r="E13">
+        <v>0.7</v>
+      </c>
+      <c r="F13" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>985</v>
+      </c>
+      <c r="B14" t="s">
+        <v>988</v>
+      </c>
+      <c r="C14" t="s">
+        <v>946</v>
+      </c>
+      <c r="D14">
+        <v>3000</v>
+      </c>
+      <c r="E14">
+        <v>0.7</v>
+      </c>
+      <c r="F14" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>985</v>
+      </c>
+      <c r="B15" t="s">
+        <v>990</v>
+      </c>
+      <c r="C15" t="s">
+        <v>950</v>
+      </c>
+      <c r="D15">
+        <v>5000</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>985</v>
+      </c>
+      <c r="B16" t="s">
+        <v>992</v>
+      </c>
+      <c r="C16" t="s">
+        <v>946</v>
+      </c>
+      <c r="D16">
+        <v>2500</v>
+      </c>
+      <c r="E16">
+        <v>0.8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>994</v>
+      </c>
+      <c r="B17" t="s">
+        <v>995</v>
+      </c>
+      <c r="C17" t="s">
+        <v>946</v>
+      </c>
+      <c r="D17">
+        <v>500</v>
+      </c>
+      <c r="E17">
+        <v>0.8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>994</v>
+      </c>
+      <c r="B18" t="s">
+        <v>997</v>
+      </c>
+      <c r="C18" t="s">
+        <v>946</v>
+      </c>
+      <c r="D18">
+        <v>1500</v>
+      </c>
+      <c r="E18">
+        <v>1.5</v>
+      </c>
+      <c r="F18" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>994</v>
+      </c>
+      <c r="B19" t="s">
+        <v>999</v>
+      </c>
+      <c r="C19" t="s">
+        <v>950</v>
+      </c>
+      <c r="D19">
+        <v>800</v>
+      </c>
+      <c r="E19">
+        <v>4.5</v>
+      </c>
+      <c r="F19" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>994</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C20" t="s">
+        <v>942</v>
+      </c>
+      <c r="D20">
+        <v>60</v>
+      </c>
+      <c r="E20">
+        <v>0.1</v>
+      </c>
+      <c r="F20" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1004</v>
+      </c>
+      <c r="C21" t="s">
+        <v>942</v>
+      </c>
+      <c r="D21">
+        <v>150</v>
+      </c>
+      <c r="E21">
+        <v>2</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B22" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C22" t="s">
+        <v>942</v>
+      </c>
+      <c r="D22">
+        <v>200</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1008</v>
+      </c>
+      <c r="C23" t="s">
+        <v>942</v>
+      </c>
+      <c r="D23">
+        <v>80</v>
+      </c>
+      <c r="E23">
+        <v>0.5</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1010</v>
+      </c>
+      <c r="C24" t="s">
+        <v>942</v>
+      </c>
+      <c r="D24">
+        <v>300</v>
+      </c>
+      <c r="E24">
+        <v>3.5</v>
+      </c>
+      <c r="F24" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B25" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C25" t="s">
+        <v>942</v>
+      </c>
+      <c r="D25">
+        <v>150</v>
+      </c>
+      <c r="E25">
+        <v>2.5</v>
+      </c>
+      <c r="F25" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B26" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C26" t="s">
+        <v>942</v>
+      </c>
+      <c r="D26">
+        <v>20</v>
+      </c>
+      <c r="E26">
+        <v>0.1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B27" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C27" t="s">
+        <v>942</v>
+      </c>
+      <c r="D27">
+        <v>40</v>
+      </c>
+      <c r="E27">
+        <v>0.1</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C28" t="s">
+        <v>946</v>
+      </c>
+      <c r="D28">
+        <v>600</v>
+      </c>
+      <c r="E28">
+        <v>0.2</v>
+      </c>
+      <c r="F28" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C29" t="s">
+        <v>942</v>
+      </c>
+      <c r="D29">
+        <v>180</v>
+      </c>
+      <c r="E29">
+        <v>0.1</v>
+      </c>
+      <c r="F29" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1024</v>
+      </c>
+      <c r="C30" t="s">
+        <v>942</v>
+      </c>
+      <c r="D30">
+        <v>120</v>
+      </c>
+      <c r="E30">
+        <v>0.2</v>
+      </c>
+      <c r="F30" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C31" t="s">
+        <v>942</v>
+      </c>
+      <c r="D31">
+        <v>30</v>
+      </c>
+      <c r="E31">
+        <v>0.2</v>
+      </c>
+      <c r="F31" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C32" t="s">
+        <v>942</v>
+      </c>
+      <c r="D32">
+        <v>180</v>
+      </c>
+      <c r="E32">
+        <v>0.3</v>
+      </c>
+      <c r="F32" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C33" t="s">
+        <v>942</v>
+      </c>
+      <c r="D33">
+        <v>60</v>
+      </c>
+      <c r="E33">
+        <v>0.6</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C34" t="s">
+        <v>942</v>
+      </c>
+      <c r="D34">
+        <v>40</v>
+      </c>
+      <c r="E34">
+        <v>0.8</v>
+      </c>
+      <c r="F34" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C35" t="s">
+        <v>942</v>
+      </c>
+      <c r="D35">
+        <v>25</v>
+      </c>
+      <c r="E35">
+        <v>0.1</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C36" t="s">
+        <v>946</v>
+      </c>
+      <c r="D36">
+        <v>800</v>
+      </c>
+      <c r="E36">
+        <v>1.3</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39CD9053-F5FB-4906-BBB6-020269F367D5}">
   <dimension ref="A1:AZ60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>

</xml_diff>